<commit_message>
update dashboard from Soccer365
</commit_message>
<xml_diff>
--- a/인천 2026 기록.xlsx
+++ b/인천 2026 기록.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://familyinter-my.sharepoint.com/personal/hwlee_familyinter_onmicrosoft_com/Documents/바탕 화면/기록/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6447" documentId="13_ncr:1_{A84C13C0-2530-4BE9-9553-B4840BB96D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFBBED24-B0B8-44E2-9F8B-6055F7649D20}"/>
+  <xr:revisionPtr revIDLastSave="7368" documentId="13_ncr:1_{A84C13C0-2530-4BE9-9553-B4840BB96D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{378D00D1-CDD2-4100-9FFA-8EE4E074696A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1770" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 토탈" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5898" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5896" uniqueCount="392">
   <si>
     <t>리그</t>
   </si>
@@ -1237,10 +1237,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>8월 16일</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>8월 23일</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -1289,7 +1285,7 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>K리그1 2026 리그순위   (2026-08-08 - 22R 진행 중)</t>
+    <t>K리그1 2026 리그순위   (2026-08-15 - 23R 진행 중)</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -5317,7 +5313,7 @@
         <v>1</v>
       </c>
       <c r="BI1" s="475" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="BJ1" s="474"/>
       <c r="BK1" s="474"/>
@@ -5715,10 +5711,10 @@
         <v>339</v>
       </c>
       <c r="BK3" s="469">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="BL3" s="469">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BM3" s="469">
         <v>5</v>
@@ -5727,17 +5723,17 @@
         <v>4</v>
       </c>
       <c r="BO3" s="469">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="BP3" s="469">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="BQ3" s="469">
         <f>BO3-BP3</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="BR3" s="469">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:77">
@@ -6319,32 +6315,32 @@
         <v>4</v>
       </c>
       <c r="BJ6" s="476" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="BK6" s="476">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="BL6" s="476">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BM6" s="476">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="BN6" s="476">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="BO6" s="476">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="BP6" s="476">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="BQ6" s="476">
         <f>BO6-BP6</f>
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="BR6" s="476">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:77">
@@ -6516,32 +6512,32 @@
         <v>5</v>
       </c>
       <c r="BJ7" s="476" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="BK7" s="476">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="BL7" s="476">
         <v>8</v>
       </c>
       <c r="BM7" s="476">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BN7" s="476">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="BO7" s="476">
         <v>25</v>
       </c>
       <c r="BP7" s="476">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="BQ7" s="476">
         <f>BO7-BP7</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="BR7" s="476">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:77">
@@ -6719,32 +6715,32 @@
         <v>6</v>
       </c>
       <c r="BJ8" s="476" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="BK8" s="476">
+        <v>23</v>
+      </c>
+      <c r="BL8" s="476">
+        <v>9</v>
+      </c>
+      <c r="BM8" s="476">
+        <v>4</v>
+      </c>
+      <c r="BN8" s="476">
+        <v>10</v>
+      </c>
+      <c r="BO8" s="476">
         <v>22</v>
       </c>
-      <c r="BL8" s="476">
-        <v>7</v>
-      </c>
-      <c r="BM8" s="476">
-        <v>9</v>
-      </c>
-      <c r="BN8" s="476">
-        <v>6</v>
-      </c>
-      <c r="BO8" s="476">
-        <v>30</v>
-      </c>
       <c r="BP8" s="476">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="BQ8" s="476">
         <f>BO8-BP8</f>
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="BR8" s="476">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:77">
@@ -6916,36 +6912,36 @@
         <f t="shared" si="12"/>
         <v>0.5</v>
       </c>
-      <c r="BI9" s="471">
+      <c r="BI9" s="476">
         <v>7</v>
       </c>
-      <c r="BJ9" s="471" t="s">
-        <v>391</v>
-      </c>
-      <c r="BK9" s="471">
-        <v>21</v>
-      </c>
-      <c r="BL9" s="471">
-        <v>8</v>
-      </c>
-      <c r="BM9" s="471">
-        <v>5</v>
-      </c>
-      <c r="BN9" s="471">
-        <v>8</v>
-      </c>
-      <c r="BO9" s="471">
-        <v>28</v>
-      </c>
-      <c r="BP9" s="471">
-        <v>24</v>
-      </c>
-      <c r="BQ9" s="471">
+      <c r="BJ9" s="476" t="s">
+        <v>353</v>
+      </c>
+      <c r="BK9" s="476">
+        <v>23</v>
+      </c>
+      <c r="BL9" s="476">
+        <v>7</v>
+      </c>
+      <c r="BM9" s="476">
+        <v>9</v>
+      </c>
+      <c r="BN9" s="476">
+        <v>7</v>
+      </c>
+      <c r="BO9" s="476">
+        <v>30</v>
+      </c>
+      <c r="BP9" s="476">
+        <v>30</v>
+      </c>
+      <c r="BQ9" s="476">
         <f>BO9-BP9</f>
-        <v>4</v>
-      </c>
-      <c r="BR9" s="471">
-        <v>29</v>
+        <v>0</v>
+      </c>
+      <c r="BR9" s="476">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:77">
@@ -7117,36 +7113,36 @@
         <f t="shared" si="12"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="BI10" s="476">
+      <c r="BI10" s="471">
         <v>8</v>
       </c>
-      <c r="BJ10" s="476" t="s">
-        <v>347</v>
-      </c>
-      <c r="BK10" s="476">
-        <v>22</v>
-      </c>
-      <c r="BL10" s="476">
+      <c r="BJ10" s="471" t="s">
+        <v>390</v>
+      </c>
+      <c r="BK10" s="471">
+        <v>21</v>
+      </c>
+      <c r="BL10" s="471">
         <v>8</v>
       </c>
-      <c r="BM10" s="476">
+      <c r="BM10" s="471">
+        <v>5</v>
+      </c>
+      <c r="BN10" s="471">
+        <v>8</v>
+      </c>
+      <c r="BO10" s="471">
+        <v>28</v>
+      </c>
+      <c r="BP10" s="471">
+        <v>24</v>
+      </c>
+      <c r="BQ10" s="471">
+        <f>BO10-BP10</f>
         <v>4</v>
       </c>
-      <c r="BN10" s="476">
-        <v>10</v>
-      </c>
-      <c r="BO10" s="476">
-        <v>20</v>
-      </c>
-      <c r="BP10" s="476">
-        <v>24</v>
-      </c>
-      <c r="BQ10" s="476">
-        <f>BO10-BP10</f>
-        <v>-4</v>
-      </c>
-      <c r="BR10" s="476">
-        <v>28</v>
+      <c r="BR10" s="471">
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:77">
@@ -7325,7 +7321,7 @@
         <v>351</v>
       </c>
       <c r="BK11" s="476">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="BL11" s="476">
         <v>6</v>
@@ -7334,17 +7330,17 @@
         <v>8</v>
       </c>
       <c r="BN11" s="476">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="BO11" s="476">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="BP11" s="476">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="BQ11" s="476">
         <f>BO11-BP11</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BR11" s="476">
         <v>26</v>
@@ -7915,7 +7911,7 @@
         <v>343</v>
       </c>
       <c r="BK14" s="472">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="BL14" s="472">
         <v>1</v>
@@ -7924,17 +7920,17 @@
         <v>8</v>
       </c>
       <c r="BN14" s="472">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BO14" s="472">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="BP14" s="472">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="BQ14" s="472">
         <f>BO14-BP14</f>
-        <v>-36</v>
+        <v>-37</v>
       </c>
       <c r="BR14" s="472">
         <v>11</v>
@@ -9107,12 +9103,8 @@
       <c r="A25" s="246" t="s">
         <v>336</v>
       </c>
-      <c r="B25" s="406" t="s">
-        <v>379</v>
-      </c>
-      <c r="C25" s="407" t="s">
-        <v>346</v>
-      </c>
+      <c r="B25" s="406"/>
+      <c r="C25" s="407"/>
       <c r="D25" s="266">
         <v>23</v>
       </c>
@@ -9195,7 +9187,7 @@
         <v>336</v>
       </c>
       <c r="B26" s="406" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C26" s="407" t="s">
         <v>346</v>
@@ -9282,7 +9274,7 @@
         <v>336</v>
       </c>
       <c r="B27" s="406" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C27" s="407" t="s">
         <v>350</v>
@@ -9369,7 +9361,7 @@
         <v>336</v>
       </c>
       <c r="B28" s="406" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C28" s="407" t="s">
         <v>346</v>
@@ -9456,7 +9448,7 @@
         <v>336</v>
       </c>
       <c r="B29" s="406" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C29" s="407" t="s">
         <v>338</v>
@@ -9543,7 +9535,7 @@
         <v>336</v>
       </c>
       <c r="B30" s="406" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C30" s="407" t="s">
         <v>362</v>
@@ -9630,7 +9622,7 @@
         <v>336</v>
       </c>
       <c r="B31" s="406" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C31" s="407" t="s">
         <v>338</v>
@@ -9717,7 +9709,7 @@
         <v>336</v>
       </c>
       <c r="B32" s="406" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C32" s="407" t="s">
         <v>346</v>
@@ -9804,10 +9796,10 @@
         <v>336</v>
       </c>
       <c r="B33" s="406" t="s">
+        <v>386</v>
+      </c>
+      <c r="C33" s="407" t="s">
         <v>387</v>
-      </c>
-      <c r="C33" s="407" t="s">
-        <v>388</v>
       </c>
       <c r="D33" s="266">
         <v>31</v>
@@ -9891,7 +9883,7 @@
         <v>336</v>
       </c>
       <c r="B34" s="406" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C34" s="407" t="s">
         <v>346</v>
@@ -9978,7 +9970,7 @@
         <v>336</v>
       </c>
       <c r="B35" s="406" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C35" s="407" t="s">
         <v>338</v>

</xml_diff>